<commit_message>
Notificación a admin además del usuario principal
</commit_message>
<xml_diff>
--- a/registro_merval.xlsx
+++ b/registro_merval.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:P11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -472,6 +472,31 @@
           <t>Semana 2 - Cierre</t>
         </is>
       </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Semana 3 - Fecha</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Semana 3 - Apertura</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Semana 3 - Máximo</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Semana 3 - Mínimo</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Semana 3 - Cierre</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -513,6 +538,23 @@
       <c r="K2" t="n">
         <v>6089.92</v>
       </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="M2" t="n">
+        <v>6094.85</v>
+      </c>
+      <c r="N2" t="n">
+        <v>6400.08</v>
+      </c>
+      <c r="O2" t="n">
+        <v>5863.46</v>
+      </c>
+      <c r="P2" t="n">
+        <v>6089.92</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -554,6 +596,23 @@
       <c r="K3" t="n">
         <v>62825</v>
       </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
+        <v>65600</v>
+      </c>
+      <c r="N3" t="n">
+        <v>66600</v>
+      </c>
+      <c r="O3" t="n">
+        <v>61800</v>
+      </c>
+      <c r="P3" t="n">
+        <v>62825</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -595,6 +654,23 @@
       <c r="K4" t="n">
         <v>4702.5</v>
       </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="M4" t="n">
+        <v>4967.5</v>
+      </c>
+      <c r="N4" t="n">
+        <v>4967.5</v>
+      </c>
+      <c r="O4" t="n">
+        <v>4500</v>
+      </c>
+      <c r="P4" t="n">
+        <v>4702.5</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -636,6 +712,23 @@
       <c r="K5" t="n">
         <v>10870</v>
       </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="M5" t="n">
+        <v>10870</v>
+      </c>
+      <c r="N5" t="n">
+        <v>11590</v>
+      </c>
+      <c r="O5" t="n">
+        <v>10200</v>
+      </c>
+      <c r="P5" t="n">
+        <v>10870</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -677,6 +770,23 @@
       <c r="K6" t="n">
         <v>667</v>
       </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="M6" t="n">
+        <v>670</v>
+      </c>
+      <c r="N6" t="n">
+        <v>708</v>
+      </c>
+      <c r="O6" t="n">
+        <v>655</v>
+      </c>
+      <c r="P6" t="n">
+        <v>667</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -718,6 +828,23 @@
       <c r="K7" t="n">
         <v>910.5</v>
       </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="M7" t="n">
+        <v>970</v>
+      </c>
+      <c r="N7" t="n">
+        <v>970</v>
+      </c>
+      <c r="O7" t="n">
+        <v>881</v>
+      </c>
+      <c r="P7" t="n">
+        <v>910.5</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -759,6 +886,23 @@
       <c r="K8" t="n">
         <v>2106</v>
       </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="M8" t="n">
+        <v>2180</v>
+      </c>
+      <c r="N8" t="n">
+        <v>2299</v>
+      </c>
+      <c r="O8" t="n">
+        <v>2085</v>
+      </c>
+      <c r="P8" t="n">
+        <v>2106</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -800,6 +944,23 @@
       <c r="K9" t="n">
         <v>1754</v>
       </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="M9" t="n">
+        <v>1869</v>
+      </c>
+      <c r="N9" t="n">
+        <v>1910</v>
+      </c>
+      <c r="O9" t="n">
+        <v>1743</v>
+      </c>
+      <c r="P9" t="n">
+        <v>1754</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -841,6 +1002,23 @@
       <c r="K10" t="n">
         <v>3270</v>
       </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="M10" t="n">
+        <v>3360</v>
+      </c>
+      <c r="N10" t="n">
+        <v>3590</v>
+      </c>
+      <c r="O10" t="n">
+        <v>3125</v>
+      </c>
+      <c r="P10" t="n">
+        <v>3270</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -880,6 +1058,23 @@
         <v>8610</v>
       </c>
       <c r="K11" t="n">
+        <v>8795</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="M11" t="n">
+        <v>9095</v>
+      </c>
+      <c r="N11" t="n">
+        <v>9640</v>
+      </c>
+      <c r="O11" t="n">
+        <v>8610</v>
+      </c>
+      <c r="P11" t="n">
         <v>8795</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualiza registro semanal del Merval
</commit_message>
<xml_diff>
--- a/registro_merval.xlsx
+++ b/registro_merval.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P11"/>
+  <dimension ref="A1:U11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -497,6 +497,31 @@
           <t>Semana 3 - Cierre</t>
         </is>
       </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Semana 4 - Fecha</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Semana 4 - Apertura</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>Semana 4 - Máximo</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>Semana 4 - Mínimo</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>Semana 4 - Cierre</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -555,6 +580,23 @@
       <c r="P2" t="n">
         <v>6089.92</v>
       </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="R2" t="n">
+        <v>6094.85</v>
+      </c>
+      <c r="S2" t="n">
+        <v>6400.08</v>
+      </c>
+      <c r="T2" t="n">
+        <v>5863.46</v>
+      </c>
+      <c r="U2" t="n">
+        <v>6089.92</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -613,6 +655,23 @@
       <c r="P3" t="n">
         <v>62825</v>
       </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="R3" t="n">
+        <v>65600</v>
+      </c>
+      <c r="S3" t="n">
+        <v>66600</v>
+      </c>
+      <c r="T3" t="n">
+        <v>61800</v>
+      </c>
+      <c r="U3" t="n">
+        <v>62825</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -671,6 +730,23 @@
       <c r="P4" t="n">
         <v>4702.5</v>
       </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="R4" t="n">
+        <v>4967.5</v>
+      </c>
+      <c r="S4" t="n">
+        <v>4967.5</v>
+      </c>
+      <c r="T4" t="n">
+        <v>4500</v>
+      </c>
+      <c r="U4" t="n">
+        <v>4702.5</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -729,6 +805,23 @@
       <c r="P5" t="n">
         <v>10870</v>
       </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="R5" t="n">
+        <v>10870</v>
+      </c>
+      <c r="S5" t="n">
+        <v>11590</v>
+      </c>
+      <c r="T5" t="n">
+        <v>10200</v>
+      </c>
+      <c r="U5" t="n">
+        <v>10870</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -787,6 +880,23 @@
       <c r="P6" t="n">
         <v>667</v>
       </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="R6" t="n">
+        <v>670</v>
+      </c>
+      <c r="S6" t="n">
+        <v>708</v>
+      </c>
+      <c r="T6" t="n">
+        <v>655</v>
+      </c>
+      <c r="U6" t="n">
+        <v>667</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -845,6 +955,23 @@
       <c r="P7" t="n">
         <v>910.5</v>
       </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="R7" t="n">
+        <v>970</v>
+      </c>
+      <c r="S7" t="n">
+        <v>970</v>
+      </c>
+      <c r="T7" t="n">
+        <v>881</v>
+      </c>
+      <c r="U7" t="n">
+        <v>910.5</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -903,6 +1030,23 @@
       <c r="P8" t="n">
         <v>2106</v>
       </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="R8" t="n">
+        <v>2180</v>
+      </c>
+      <c r="S8" t="n">
+        <v>2299</v>
+      </c>
+      <c r="T8" t="n">
+        <v>2085</v>
+      </c>
+      <c r="U8" t="n">
+        <v>2106</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -961,6 +1105,23 @@
       <c r="P9" t="n">
         <v>1754</v>
       </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="R9" t="n">
+        <v>1869</v>
+      </c>
+      <c r="S9" t="n">
+        <v>1910</v>
+      </c>
+      <c r="T9" t="n">
+        <v>1743</v>
+      </c>
+      <c r="U9" t="n">
+        <v>1754</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1019,6 +1180,23 @@
       <c r="P10" t="n">
         <v>3270</v>
       </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="R10" t="n">
+        <v>3360</v>
+      </c>
+      <c r="S10" t="n">
+        <v>3590</v>
+      </c>
+      <c r="T10" t="n">
+        <v>3125</v>
+      </c>
+      <c r="U10" t="n">
+        <v>3270</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1075,6 +1253,23 @@
         <v>8610</v>
       </c>
       <c r="P11" t="n">
+        <v>8795</v>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="R11" t="n">
+        <v>9095</v>
+      </c>
+      <c r="S11" t="n">
+        <v>9640</v>
+      </c>
+      <c r="T11" t="n">
+        <v>8610</v>
+      </c>
+      <c r="U11" t="n">
         <v>8795</v>
       </c>
     </row>

</xml_diff>